<commit_message>
Checkpoint before backlog analytic study
</commit_message>
<xml_diff>
--- a/scripts/reports/qa_d_projetos.xlsx
+++ b/scripts/reports/qa_d_projetos.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="d_Projetos" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="prefixo_conflicts" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="missing_prefix" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="backlog_sem_controle" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="producao_sem_controle" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sem_chave" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="idp_overrides" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="d_Projetos" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="prefixo_conflicts" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="missing_prefix" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="backlog_sem_controle" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="producao_sem_controle" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="sem_chave" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="idp_overrides" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="cliente_overrides" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -431,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E52"/>
+  <dimension ref="A1:E68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -509,19 +510,15 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2020-001-01</t>
+          <t>2019-262-01</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>C. AERONÁUTICA</t>
-        </is>
-      </c>
+          <t>618/21</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
@@ -530,24 +527,20 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2022-051-03</t>
+          <t>2020-001-01</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>845/24</t>
+          <t>001/20</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>PRODAM SP - Lote 3</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>PMSP/SMG/PROD</t>
-        </is>
-      </c>
+          <t>C. AERONÁUTICA</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -555,22 +548,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2022-134-01</t>
+          <t>2022-051-03</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>018/23</t>
+          <t>845/24</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>MPF (SDWAN) - 2022-134-01</t>
+          <t>PRODAM SP - Lote 3</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>MPF</t>
+          <t>PMSP/SMG/PROD</t>
         </is>
       </c>
     </row>
@@ -580,22 +573,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2023-061-01</t>
+          <t>2022-134-01</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>105/24</t>
+          <t>018/23</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>SEPLAD-DF BLD + Anti-DDoS 2024</t>
+          <t>MPF (SDWAN) - 2022-134-01</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>MPF</t>
         </is>
       </c>
     </row>
@@ -605,12 +598,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2023-286-01</t>
+          <t>2022-318-01</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>41/23</t>
+          <t>8/23</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
@@ -622,22 +615,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2023-303-01</t>
+          <t>2023-061-01</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>113/24</t>
+          <t>105/24</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>BB - SDWan</t>
+          <t>SEPLAD-DF BLD + Anti-DDoS 2024</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>BCO BRASIL</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -647,20 +640,24 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2023-549-01</t>
+          <t>2023-286-01</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>549</t>
+          <t>41/23</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>SESI/ SENAI - SP</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr"/>
+          <t>ECT</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>ECT</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -668,22 +665,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2023-549-03</t>
+          <t>2023-303-01</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>549</t>
+          <t>113/24</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>SESI SERVICO SOCIAL DA INDUSTRIA</t>
+          <t>BB - SDWan</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>BCO BRASIL</t>
         </is>
       </c>
     </row>
@@ -693,24 +690,16 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2023-623-02</t>
+          <t>2023-516-01</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>1078/25</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>SEFA-PA - SDWAN</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>SEFA PARA</t>
-        </is>
-      </c>
+          <t>107/24</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -718,24 +707,20 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2023-694-02</t>
+          <t>2023-549-01</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>119/24</t>
+          <t>549/23</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Pref. do RIO - Adm. Indireta</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>PREF RIO ADM INDIRETA</t>
-        </is>
-      </c>
+          <t>SESI/ SENAI - SP</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -743,22 +728,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2023-810-02</t>
+          <t>2023-623-02</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>118/24</t>
+          <t>1078/25</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>MARINHA - SDWAN</t>
+          <t>SEFA-PA - SDWAN</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>C MARINHA</t>
+          <t>SEFA PARA</t>
         </is>
       </c>
     </row>
@@ -768,22 +753,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2023-934-01</t>
+          <t>2023-694-02</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>875/25</t>
+          <t>694/23</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>CEF - Integrador</t>
+          <t>Pref. do RIO - Adm. Indireta</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>CEF</t>
+          <t>PREF RIO ADM INDIRETA</t>
         </is>
       </c>
     </row>
@@ -793,24 +778,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2023-948-02</t>
+          <t>2023-761-01</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>120/24</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Pref. do RIO - Adm. Direta</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>PREF RIO ADM DIRETA</t>
-        </is>
-      </c>
+          <t>104/24</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -818,20 +795,24 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2024-0253-01</t>
+          <t>2023-810-02</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>0253</t>
+          <t>810/23</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>SEPLAG-MG</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr"/>
+          <t>MARINHA - SDWAN</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>C MARINHA</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -839,19 +820,15 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2024-0692-02</t>
+          <t>2023-833-01</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>0692</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>CONAB</t>
-        </is>
-      </c>
+          <t>103/24</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr"/>
     </row>
     <row r="19">
@@ -860,20 +837,24 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2024-1012-01</t>
+          <t>2023-934-01</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>1012</t>
+          <t>875/25</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>SANEPAR</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr"/>
+          <t>CEF - Integrador</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>CEF</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -881,22 +862,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2024-1092-01</t>
+          <t>2023-948-02</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>1092</t>
+          <t>948/23</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>COMAER - CINDACTA III REDE DET</t>
+          <t>Pref. do RIO - Adm. Direta</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>C AERONAUTICA</t>
+          <t>PREF RIO ADM DIRETA</t>
         </is>
       </c>
     </row>
@@ -906,24 +887,16 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2024-1253-01</t>
+          <t>2023-983-01</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>1253</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>COMAER - CINDACTA I - REDE DET</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>C AERONAUTICA</t>
-        </is>
-      </c>
+          <t>109/24</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -931,24 +904,16 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2024-1310-02</t>
+          <t>2023-996-0</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>1168/25</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>DPU</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>DEF.PUB.UNIAO</t>
-        </is>
-      </c>
+          <t>115/24</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -956,12 +921,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2024-253-01</t>
+          <t>2024-0253-01</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>1067/25</t>
+          <t>0253/24</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -969,11 +934,7 @@
           <t>SEPLAG-MG</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>SEPLAG MG</t>
-        </is>
-      </c>
+      <c r="E23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -981,12 +942,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2024-383-01</t>
+          <t>2024-0383-01</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>1165/25</t>
+          <t>0383/24</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -994,11 +955,7 @@
           <t>TRE-MG 2025</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>TRE MG</t>
-        </is>
-      </c>
+      <c r="E24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1006,24 +963,20 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2024-597-01</t>
+          <t>2024-0383-02</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>737/24</t>
+          <t>0383/24</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>SEDUC MS</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>SED MS</t>
-        </is>
-      </c>
+          <t>TRE-MG 2025</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1031,16 +984,24 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2024-598-01</t>
+          <t>2024-0692-02</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>1007/25</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
+          <t>1203/26</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>CONAB</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>C O N A B</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1048,24 +1009,20 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2024-692-01</t>
+          <t>2024-1012-01</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>1203/26</t>
+          <t>1012/24</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>CONAB</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>C O N A B</t>
-        </is>
-      </c>
+          <t>SANEPAR</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1073,17 +1030,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2024-971-02</t>
+          <t>2024-1092-01</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>1199/25</t>
+          <t>1092/24</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>AERONÁUTICA - CRCEA-SE</t>
+          <t>COMAER - CINDACTA III REDE DET</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1098,22 +1055,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2024-998-01</t>
+          <t>2024-1253-01</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>1066/25</t>
+          <t>1275/26</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>TJ-TO</t>
+          <t>COMAER - CINDACTA I - REDE DET</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>3173154</t>
+          <t>C AERONAUTICA</t>
         </is>
       </c>
     </row>
@@ -1123,24 +1080,16 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2025-0013-01</t>
+          <t>2024-1253-02</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>1198/25</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>SEFAZ-AM</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>SEFAZ-AM</t>
-        </is>
-      </c>
+          <t>1275/26</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1148,22 +1097,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2025-0026-01</t>
+          <t>2024-1310-02</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>0026</t>
+          <t>1168/25</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>COMAER REDE ATN  (CI, CII, CIII, CIV E CRCEA-SE)</t>
+          <t>DPU</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>C AERONAUTICA</t>
+          <t>DEF.PUB.UNIAO</t>
         </is>
       </c>
     </row>
@@ -1173,16 +1122,24 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2025-0026-02</t>
+          <t>2024-253-01</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>1190/25</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr"/>
+          <t>1067/25</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>SEPLAG-MG</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>SEPLAG MG</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1190,22 +1147,22 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2025-0155-01</t>
+          <t>2024-383-01</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>1230/26</t>
+          <t>1165/25</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>MP ES SDWAN</t>
+          <t>TRE-MG 2025</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>MIN. PUB. ES</t>
+          <t>TRE MG</t>
         </is>
       </c>
     </row>
@@ -1215,22 +1172,22 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2025-0215-02</t>
+          <t>2024-597-01</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>1125/25</t>
+          <t>737/24</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>STJ</t>
+          <t>SEDUC MS</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SED MS</t>
         </is>
       </c>
     </row>
@@ -1240,22 +1197,22 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2025-0216-01</t>
+          <t>2024-597-02</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>0216</t>
+          <t>597/24</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>PRODEMGE SDWAN</t>
+          <t>SEDUC MS - ADITIVO</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>PRODEMGE</t>
+          <t>SEDUC MS</t>
         </is>
       </c>
     </row>
@@ -1265,24 +1222,16 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2025-0229-01</t>
+          <t>2024-598-01</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>0229</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>SANEPAR</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>SANEPAR</t>
-        </is>
-      </c>
+          <t>1007/25</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1290,22 +1239,22 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2025-0339-01</t>
+          <t>2024-692-01</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>1175/25</t>
+          <t>1203/26</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>TSE - BLD Sdwan</t>
+          <t>CONAB</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>T.S.E.</t>
+          <t>C O N A B</t>
         </is>
       </c>
     </row>
@@ -1315,22 +1264,22 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2025-0365-01</t>
+          <t>2024-971-02</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>1049/25</t>
+          <t>1199/25</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>BANCO DO BRASIL REPAR</t>
+          <t>AERONÁUTICA - CRCEA-SE</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>BCO BRASIL</t>
+          <t>C AERONAUTICA</t>
         </is>
       </c>
     </row>
@@ -1340,22 +1289,22 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2025-0378-01</t>
+          <t>2024-998-01</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>1205/25</t>
+          <t>1066/25</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>MPGO - UCC</t>
+          <t>TJ-TO</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>GOIAS MP PROC</t>
+          <t>3173154</t>
         </is>
       </c>
     </row>
@@ -1365,22 +1314,22 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2025-0407-01</t>
+          <t>2025-0013-01</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>1227/25</t>
+          <t>1198/25</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>FUNDAÇÃO DO ABC</t>
+          <t>SEFAZ-AM</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>FUND.ABC</t>
+          <t>SEFAZ-AM</t>
         </is>
       </c>
     </row>
@@ -1390,22 +1339,22 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2025-0446-01</t>
+          <t>2025-0026-01</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>1108/25</t>
+          <t>0026/25</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>SERPRO</t>
+          <t>COMAER REDE ATN  (CI, CII, CIII, CIV E CRCEA-SE)</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>SERPRO</t>
+          <t>C AERONAUTICA</t>
         </is>
       </c>
     </row>
@@ -1415,24 +1364,16 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2025-0588-01</t>
+          <t>2025-0026-02</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>0588</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>CÂMARA DOS DEPUTADOS</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+          <t>1190/25</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -1440,24 +1381,16 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2025-0598-01</t>
+          <t>2025-0046-01</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>1094/25</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>SEDUC RS</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>SEC RS</t>
-        </is>
-      </c>
+          <t>1293/26</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -1465,22 +1398,22 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2025-0599-01</t>
+          <t>2025-0155-01</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>0599</t>
+          <t>1230/26</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>TRE-SP</t>
+          <t>MP ES SDWAN</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>TRE-SP</t>
+          <t>MIN. PUB. ES</t>
         </is>
       </c>
     </row>
@@ -1490,22 +1423,22 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2025-0643-01</t>
+          <t>2025-0215-02</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>1249/26</t>
+          <t>1125/25</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>COMPANHIA DOCAS DO PARA</t>
+          <t>STJ</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>CDP</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -1515,22 +1448,22 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2025-0698-01</t>
+          <t>2025-0216-01</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>0698</t>
+          <t>0216/25</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>PRODEST ES</t>
+          <t>PRODEMGE SDWAN</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>PRODEMGE</t>
         </is>
       </c>
     </row>
@@ -1540,22 +1473,22 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2025-0813-01</t>
+          <t>2025-0229-01</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>0813</t>
+          <t>0229/25</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>BANCO DO BRASIL REDE MAN SP</t>
+          <t>SANEPAR</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>BANCO DO BRASIL</t>
+          <t>SANEPAR</t>
         </is>
       </c>
     </row>
@@ -1565,22 +1498,22 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2025-0971-01</t>
+          <t>2025-0339-01</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>0971</t>
+          <t>1175/25</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>CESAN</t>
+          <t>TSE - BLD Sdwan</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>CESAN</t>
+          <t>T.S.E.</t>
         </is>
       </c>
     </row>
@@ -1590,22 +1523,22 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2025-1213-01</t>
+          <t>2025-0365-01</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>1213</t>
+          <t>1049/25</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>TRF-1 MPLS SDWAN</t>
+          <t>BANCO DO BRASIL REPAR</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>TRF1</t>
+          <t>BCO BRASIL</t>
         </is>
       </c>
     </row>
@@ -1615,22 +1548,22 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-0010-01</t>
+          <t>2025-0378-01</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>0010</t>
+          <t>1205/25</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>HCFMUSP TSIP</t>
+          <t>MPGO - UCC</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>HCFMUSP</t>
+          <t>GOIAS MP PROC</t>
         </is>
       </c>
     </row>
@@ -1640,20 +1573,24 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-0025-0</t>
+          <t>2025-0407-01</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>0025</t>
+          <t>1227/25</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>BASA Multisserviço MPLS + Dedicada</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr"/>
+          <t>FUNDAÇÃO DO ABC</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>FUND.ABC</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -1661,22 +1598,414 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
+          <t>2025-0446-01</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>1108/25</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>SERPRO</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>SERPRO</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>2025-0588-01</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>0588/25</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>CÂMARA DOS DEPUTADOS</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>2025-0598-01</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>1094/25</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>SEDUC RS</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>SEC RS</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>2025-0599-01</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>1312/26</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>TRE-SP</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>TRE-SP</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>2025-0643-01</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>1249/26</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>COMPANHIA DOCAS DO PARA</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>CDP</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>2025-0698-01</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>0698/25</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>PRODEST ES</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>2025-0729-02</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>1316/26</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>MPM - UCC e VOZ</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>MPU</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>2025-0796-02</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>0796/25</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>PRODESP dwdm</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>PRODESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>2025-0813-01</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>0813/25</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>BANCO DO BRASIL REDE MAN SP</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>BANCO DO BRASIL</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>2025-0971-01</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>0971/25</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>CESAN</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>CESAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>2025-1213-01</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>1213/25</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>TRF-1 MPLS SDWAN</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>TRF1</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>2025-1293-01</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>1293/25</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>TSE (BLD + Anti-DDoS)</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>TSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>2026-0010-01</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>0010/26</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>HCFMUSP TSIP</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>HCFMUSP</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
           <t>2026-0025-01</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>0025</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>0025/26</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
         <is>
           <t>BASA Multisserviço MPLS + Dedicada</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr">
+      <c r="E65" t="inlineStr">
         <is>
           <t>BASA</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>2026-0042-01</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>1313/26</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr"/>
+      <c r="E66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>2026-0114-01</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>0114/26</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>COMAER INTRAER - PAME RJ</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>C AERONAUTICA</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>2026-0147-01</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>0147/26</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>TCTA EPL L2L</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>TCTA</t>
         </is>
       </c>
     </row>
@@ -1691,7 +2020,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1709,7 +2038,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0025</t>
+          <t>0383/24</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -1719,10 +2048,30 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>549</t>
+          <t>1203/26</t>
         </is>
       </c>
       <c r="B3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>1275/26</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>597/24</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1768,7 +2117,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1796,42 +2145,42 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2023-286-01</t>
+          <t>2025-0046-01</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>41/23</t>
+          <t>1293/26</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0000-1030-01</t>
+          <t>2023-286-01</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>1157/25</t>
+          <t>41/23</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2025-0026-02</t>
+          <t>0000-1030-01</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1190/25</t>
+          <t>1157/25</t>
         </is>
       </c>
     </row>
@@ -1845,7 +2194,7 @@
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>1194/25</t>
+          <t>1190/25</t>
         </is>
       </c>
     </row>
@@ -1859,7 +2208,7 @@
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>1219/26</t>
+          <t>1194/25</t>
         </is>
       </c>
     </row>
@@ -1873,7 +2222,99 @@
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>1255/26</t>
+          <t>1219/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2024-1253-02</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>1275/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2025-0046-01</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>1293/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>0000-1030-01</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>1157/25</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2024-1253-02</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>1240/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-0042-01</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>1313/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2023-286-01</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ECT</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>ECT</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>41/23</t>
         </is>
       </c>
     </row>
@@ -1888,7 +2329,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1944,12 +2385,48 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2024-598-01</t>
+          <t>0000-1030-01</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
+        <is>
+          <t>1157/25</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2023-286-01</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ECT</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ECT</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>41/23</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2024-598-01</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
         <is>
           <t>1007/25</t>
         </is>
@@ -2040,6 +2517,68 @@
       <c r="B4" t="inlineStr">
         <is>
           <t>2024-692-01</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>carimbo_prefixo</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>cliente</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t># Formato: prefixo/ano</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>NOME DO CLIENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t># 103/24</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>BANCO DO BRASIL</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t># 41/23</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>CAIXA ECONOMICA FEDERAL</t>
         </is>
       </c>
     </row>
@@ -2304,13 +2843,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{59603094-72EC-4074-A88F-2A982E70066C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6EB5A7D8-2DD1-4E70-A00F-C60A1D4FA489}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{84505E78-421B-4E9E-AB78-244956C79674}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2772056D-58D3-41E2-8D9C-607DD349A083}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C3BFF3E-3FD6-4087-8572-26EEDFBA4A85}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EB473F58-92C9-4B3E-AD36-CCB65CAC01AB}"/>
 </file>
</xml_diff>